<commit_message>
Add student balances report with localized Excel export
</commit_message>
<xml_diff>
--- a/payments_report_ru.xlsx
+++ b/payments_report_ru.xlsx
@@ -1,36 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="true" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="11_FD21BF15A05EB549FB4E599476A8462122E1F548" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{254F84C4-AB00-4C24-829F-65844D70C3B9}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Платежи" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="122211"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="31">
   <si>
     <t>Отчёт по платежам</t>
   </si>
   <si>
-    <t>С</t>
-  </si>
-  <si>
     <t>2026-07-01</t>
   </si>
   <si>
-    <t>По</t>
-  </si>
-  <si>
-    <t>2026-08-31</t>
-  </si>
-  <si>
     <t>Всего платежей</t>
   </si>
   <si>
@@ -110,23 +107,30 @@
   </si>
   <si>
     <t>Частичная оплата за август</t>
+  </si>
+  <si>
+    <t>С 2026-07-01</t>
+  </si>
+  <si>
+    <t>По 2026-08-31</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color/>
     </font>
   </fonts>
   <fills count="2">
@@ -137,7 +141,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -145,26 +149,52 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="false">
-      <alignment/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -420,160 +450,190 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col customWidth="true" max="2" min="1" width="18"/>
-    <col customWidth="true" max="5" min="3" width="24"/>
-    <col customWidth="true" max="8" min="6" width="18"/>
-    <col customWidth="true" max="9" min="9" width="42"/>
+    <col min="1" max="1" width="14.88671875" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="5" width="24" customWidth="1"/>
+    <col min="6" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="42" customWidth="1"/>
+    <col min="11" max="11" width="12.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
     </row>
-    <row r="2">
-      <c r="A2" t="s">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="J6" s="2"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
+      <c r="C7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="J7" s="2"/>
     </row>
-    <row r="4">
-      <c r="A4" t="s">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B4">
-        <v>2</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" t="s">
-        <v>9</v>
-      </c>
-      <c r="H4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I4" t="s">
-        <v>11</v>
-      </c>
-      <c r="J4" t="s">
-        <v>10</v>
-      </c>
-      <c r="K4" t="s">
-        <v>12</v>
-      </c>
-      <c r="L4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" t="s">
-        <v>2</v>
-      </c>
-      <c r="C7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G7" t="s">
-        <v>27</v>
-      </c>
-      <c r="H7" t="s">
-        <v>8</v>
-      </c>
-      <c r="I7" t="s">
+      <c r="I8" s="2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8" t="s">
-        <v>25</v>
-      </c>
-      <c r="F8" t="s">
-        <v>30</v>
-      </c>
-      <c r="G8" t="s">
-        <v>27</v>
-      </c>
-      <c r="H8" t="s">
-        <v>8</v>
-      </c>
-      <c r="I8" t="s">
-        <v>31</v>
-      </c>
+      <c r="J8" s="2"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>